<commit_message>
data(swarm-disaster): G09-P3-B6 verify Sora and visual QA
</commit_message>
<xml_diff>
--- a/config/swarm-disaster/data/SwarmDisasterProgression.xlsx
+++ b/config/swarm-disaster/data/SwarmDisasterProgression.xlsx
@@ -575,7 +575,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="30" customWidth="1" style="5" min="2" max="3"/>
     <col width="37" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="17" customWidth="1" style="5" min="5" max="8"/>
@@ -3455,7 +3455,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="32" customWidth="1" style="5" min="2" max="3"/>
     <col width="43" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="19" customWidth="1" style="5" min="5" max="8"/>
@@ -13856,7 +13856,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="32" customWidth="1" style="5" min="2" max="3"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="26" customWidth="1" style="5" min="5" max="8"/>
@@ -22658,7 +22658,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="33" customWidth="1" style="5" min="2" max="3"/>
     <col width="44" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="20" customWidth="1" style="5" min="5" max="8"/>
@@ -24871,7 +24871,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="30" customWidth="1" style="5" min="2" max="3"/>
     <col width="37" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="22" customWidth="1" style="5" min="5" max="8"/>
@@ -25975,7 +25975,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="33" customWidth="1" style="5" min="2" max="3"/>
     <col width="40" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="20" customWidth="1" style="5" min="5" max="8"/>
@@ -29835,7 +29835,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="33" customWidth="1" style="5" min="2" max="3"/>
     <col width="38" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="20" customWidth="1" style="5" min="5" max="8"/>
@@ -31077,7 +31077,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="30" customWidth="1" style="5" min="2" max="3"/>
     <col width="51" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="26" customWidth="1" style="5" min="5" max="8"/>
@@ -36971,7 +36971,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="33" customWidth="1" style="5" min="2" max="3"/>
     <col width="36" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="20" customWidth="1" style="5" min="5" max="8"/>
@@ -43379,7 +43379,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="32" customWidth="1" style="5" min="2" max="3"/>
     <col width="45" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="28" customWidth="1" style="5" min="5" max="8"/>
@@ -48443,7 +48443,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="26" customWidth="1" style="5" min="2" max="3"/>
     <col width="41" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="22" customWidth="1" style="5" min="5" max="8"/>
@@ -54539,7 +54539,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="28" customWidth="1" style="5" min="2" max="3"/>
     <col width="42" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="22" customWidth="1" style="5" min="5" max="8"/>
@@ -57877,7 +57877,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" style="5" min="2" max="3"/>
+    <col width="32" customWidth="1" style="5" min="2" max="3"/>
     <col width="53" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" style="5" min="4" max="4"/>
     <col width="28" customWidth="1" style="5" min="5" max="8"/>

</xml_diff>